<commit_message>
Working, but need to implement load two sheet into baseline and combine baseline and table8
</commit_message>
<xml_diff>
--- a/data/sample.xlsx
+++ b/data/sample.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dskin\Documents\Projects\propensity_score_matching\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9815A95A-852D-413C-9D2E-02A640BCDD98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE640C1B-1E33-4BDD-9785-03504315C490}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-14505" yWindow="-720" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{8D6ADBF5-96F6-B143-86A8-5692DBE5BF1C}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="777" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="772" uniqueCount="263">
   <si>
     <t>dob</t>
   </si>
@@ -311,9 +311,6 @@
   </si>
   <si>
     <t xml:space="preserve">silicone </t>
-  </si>
-  <si>
-    <t>300 (R), 400 (L)</t>
   </si>
   <si>
     <t>III</t>
@@ -770,16 +767,10 @@
     <t>expander removal and debridement</t>
   </si>
   <si>
-    <t>275 (R) 295 (L)</t>
-  </si>
-  <si>
     <t>lymphedema</t>
   </si>
   <si>
     <t>capsulotomy and fat grafting</t>
-  </si>
-  <si>
-    <t>465 (R) 235 (L)</t>
   </si>
   <si>
     <r>
@@ -845,9 +836,6 @@
     <t>0.1 mm</t>
   </si>
   <si>
-    <t>300 (R) 400 (L)</t>
-  </si>
-  <si>
     <t>plan to swap for saline</t>
   </si>
   <si>
@@ -957,9 +945,6 @@
   </si>
   <si>
     <t>6mm x 2mm )(IDC), 9 cm DCIS</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 300 (R) 200 (L)</t>
   </si>
   <si>
     <r>
@@ -1787,7 +1772,7 @@
         <v>18</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="D1" s="9" t="s">
         <v>20</v>
@@ -1823,7 +1808,7 @@
         <v>78</v>
       </c>
       <c r="O1" s="14" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="P1" s="9" t="s">
         <v>6</v>
@@ -1841,7 +1826,7 @@
         <v>3</v>
       </c>
       <c r="U1" s="9" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="V1" s="9" t="s">
         <v>41</v>
@@ -1853,19 +1838,19 @@
         <v>42</v>
       </c>
       <c r="Y1" s="9" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="Z1" s="9" t="s">
         <v>24</v>
       </c>
       <c r="AA1" s="9" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="AB1" s="9" t="s">
         <v>43</v>
       </c>
       <c r="AC1" s="15" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="AD1" s="15" t="s">
         <v>11</v>
@@ -1874,7 +1859,7 @@
         <v>60</v>
       </c>
       <c r="AF1" s="9" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="AG1" s="9" t="s">
         <v>28</v>
@@ -1954,14 +1939,14 @@
         <v>70</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E2" s="12">
         <v>28835</v>
       </c>
       <c r="F2" s="18">
         <f ca="1">YEARFRAC(E2,TODAY())</f>
-        <v>47.222222222222221</v>
+        <v>47.225000000000001</v>
       </c>
       <c r="G2" s="20">
         <v>20.09</v>
@@ -2049,7 +2034,7 @@
         <v>0</v>
       </c>
       <c r="AJ2" s="18" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AK2" s="18">
         <v>2</v>
@@ -2058,13 +2043,13 @@
         <v>0</v>
       </c>
       <c r="AM2" s="32" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="AN2" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="AO2" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AP2" s="1">
         <v>0</v>
@@ -2076,7 +2061,7 @@
         <v>50</v>
       </c>
       <c r="AS2" s="27" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="AT2" s="27"/>
       <c r="AU2" s="27"/>
@@ -2102,23 +2087,23 @@
     </row>
     <row r="3" spans="1:54">
       <c r="A3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B3" s="2">
         <v>43868</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E3" s="2">
         <v>30389</v>
       </c>
       <c r="F3" s="18">
         <f t="shared" ref="F3:F20" ca="1" si="0">YEARFRAC(E3,TODAY())</f>
-        <v>42.963888888888889</v>
+        <v>42.966666666666669</v>
       </c>
       <c r="G3" s="5">
         <v>24.72</v>
@@ -2191,22 +2176,22 @@
         <v>1</v>
       </c>
       <c r="AE3" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AF3" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AG3" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AH3" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AI3" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AJ3" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AK3" s="3">
         <v>2</v>
@@ -2215,13 +2200,13 @@
         <v>0</v>
       </c>
       <c r="AM3" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AN3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AO3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AP3">
         <v>0</v>
@@ -2233,7 +2218,7 @@
         <v>54</v>
       </c>
       <c r="AV3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="AW3" s="28">
         <v>0</v>
@@ -2262,14 +2247,14 @@
         <v>70</v>
       </c>
       <c r="D4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E4" s="2">
         <v>31680</v>
       </c>
       <c r="F4" s="18">
         <f t="shared" ca="1" si="0"/>
-        <v>39.43333333333333</v>
+        <v>39.43611111111111</v>
       </c>
       <c r="G4" s="5">
         <v>22.87</v>
@@ -2357,7 +2342,7 @@
         <v>0</v>
       </c>
       <c r="AJ4" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AK4" s="3">
         <v>2</v>
@@ -2366,13 +2351,13 @@
         <v>0</v>
       </c>
       <c r="AM4" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="AN4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="AO4" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="AP4">
         <v>0</v>
@@ -2384,10 +2369,10 @@
         <v>50</v>
       </c>
       <c r="AS4" s="28" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="AT4" s="28" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="AU4" s="28" t="s">
         <v>67</v>
@@ -2399,7 +2384,7 @@
         <v>1</v>
       </c>
       <c r="AX4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="AY4">
         <v>1</v>
@@ -2422,17 +2407,17 @@
         <v>44048</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="D5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E5" s="2">
         <v>23434</v>
       </c>
       <c r="F5" s="18">
         <f t="shared" ca="1" si="0"/>
-        <v>62.011111111111113</v>
+        <v>62.013888888888886</v>
       </c>
       <c r="G5" s="5">
         <v>24.57</v>
@@ -2520,7 +2505,7 @@
         <v>0</v>
       </c>
       <c r="AJ5" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AK5" s="3">
         <v>1</v>
@@ -2529,13 +2514,13 @@
         <v>1</v>
       </c>
       <c r="AM5" s="3" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="AN5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AO5" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AP5">
         <v>0</v>
@@ -2547,19 +2532,19 @@
         <v>50</v>
       </c>
       <c r="AS5" s="28" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="AT5" s="28" t="s">
         <v>63</v>
       </c>
       <c r="AV5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AW5" s="28">
         <v>1</v>
       </c>
       <c r="AX5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="AY5">
         <v>1</v>
@@ -2579,17 +2564,17 @@
         <v>44127</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="D6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E6" s="2">
         <v>24739</v>
       </c>
       <c r="F6" s="18">
         <f t="shared" ca="1" si="0"/>
-        <v>58.43611111111111</v>
+        <v>58.43888888888889</v>
       </c>
       <c r="G6" s="5">
         <v>17.78</v>
@@ -2617,7 +2602,7 @@
         <v>0</v>
       </c>
       <c r="P6" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="Q6" s="3">
         <v>1</v>
@@ -2668,31 +2653,31 @@
         <v>0</v>
       </c>
       <c r="AG6" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AH6" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AI6" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AJ6" s="25" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AK6" s="3">
         <v>2</v>
       </c>
       <c r="AL6" s="25" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AM6" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AN6" s="16" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AO6" s="16" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AP6">
         <v>0</v>
@@ -2710,7 +2695,7 @@
         <v>1</v>
       </c>
       <c r="AX6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="AY6">
         <v>1</v>
@@ -2736,14 +2721,14 @@
         <v>70</v>
       </c>
       <c r="D7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E7" s="2">
         <v>32050</v>
       </c>
       <c r="F7" s="18">
         <f t="shared" ca="1" si="0"/>
-        <v>38.419444444444444</v>
+        <v>38.422222222222224</v>
       </c>
       <c r="G7" s="5">
         <v>21.96</v>
@@ -2831,7 +2816,7 @@
         <v>0</v>
       </c>
       <c r="AJ7" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AK7" s="3">
         <v>2</v>
@@ -2840,13 +2825,13 @@
         <v>1</v>
       </c>
       <c r="AM7" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="AN7" t="s">
+        <v>126</v>
+      </c>
+      <c r="AO7" t="s">
         <v>127</v>
-      </c>
-      <c r="AO7" t="s">
-        <v>128</v>
       </c>
       <c r="AP7">
         <v>0</v>
@@ -2858,7 +2843,7 @@
         <v>54</v>
       </c>
       <c r="AS7" s="28" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="AV7">
         <v>0</v>
@@ -2881,23 +2866,23 @@
     </row>
     <row r="8" spans="1:54">
       <c r="A8" s="16" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B8" s="2">
         <v>44169</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="D8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E8" s="2">
         <v>30752</v>
       </c>
       <c r="F8" s="18">
         <f t="shared" ca="1" si="0"/>
-        <v>41.972222222222221</v>
+        <v>41.975000000000001</v>
       </c>
       <c r="G8" s="5">
         <v>21.97</v>
@@ -2970,37 +2955,37 @@
         <v>1</v>
       </c>
       <c r="AE8" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AF8" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AG8" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AH8" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AI8" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AJ8" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AK8" s="3">
         <v>2</v>
       </c>
       <c r="AL8" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AM8" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AN8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AO8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AP8">
         <v>0</v>
@@ -3015,13 +3000,13 @@
         <v>63</v>
       </c>
       <c r="AV8" t="s">
+        <v>129</v>
+      </c>
+      <c r="AW8" s="28">
+        <v>1</v>
+      </c>
+      <c r="AX8" t="s">
         <v>130</v>
-      </c>
-      <c r="AW8" s="28">
-        <v>1</v>
-      </c>
-      <c r="AX8" t="s">
-        <v>131</v>
       </c>
       <c r="AY8">
         <v>0</v>
@@ -3047,14 +3032,14 @@
         <v>70</v>
       </c>
       <c r="D9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E9" s="2">
         <v>34748</v>
       </c>
       <c r="F9" s="18">
         <f t="shared" ca="1" si="0"/>
-        <v>31.036111111111111</v>
+        <v>31.038888888888888</v>
       </c>
       <c r="G9" s="5">
         <v>22.31</v>
@@ -3142,7 +3127,7 @@
         <v>1</v>
       </c>
       <c r="AJ9" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AK9" s="3">
         <v>0</v>
@@ -3151,13 +3136,13 @@
         <v>0</v>
       </c>
       <c r="AM9" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="AN9" s="6" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="AO9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="AP9">
         <v>0</v>
@@ -3195,17 +3180,17 @@
         <v>44141</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="D10" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E10" s="2">
         <v>23602</v>
       </c>
       <c r="F10" s="18">
         <f t="shared" ca="1" si="0"/>
-        <v>61.55</v>
+        <v>61.552777777777777</v>
       </c>
       <c r="G10" s="5">
         <v>19.91</v>
@@ -3293,7 +3278,7 @@
         <v>0</v>
       </c>
       <c r="AJ10" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AK10" s="3">
         <v>2</v>
@@ -3305,10 +3290,10 @@
         <v>0</v>
       </c>
       <c r="AN10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AO10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AP10">
         <v>0</v>
@@ -3320,10 +3305,10 @@
         <v>54</v>
       </c>
       <c r="AS10" s="28" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="AV10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AW10" s="28">
         <v>0</v>
@@ -3352,14 +3337,14 @@
         <v>70</v>
       </c>
       <c r="D11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E11" s="2">
         <v>31680</v>
       </c>
       <c r="F11" s="18">
         <f t="shared" ca="1" si="0"/>
-        <v>39.43333333333333</v>
+        <v>39.43611111111111</v>
       </c>
       <c r="G11" s="5">
         <v>22.87</v>
@@ -3447,7 +3432,7 @@
         <v>0</v>
       </c>
       <c r="AJ11" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AK11" s="3">
         <v>2</v>
@@ -3456,13 +3441,13 @@
         <v>0</v>
       </c>
       <c r="AM11" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="AN11" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="AO11" s="6" t="s">
         <v>140</v>
-      </c>
-      <c r="AO11" s="6" t="s">
-        <v>141</v>
       </c>
       <c r="AP11">
         <v>0</v>
@@ -3474,10 +3459,10 @@
         <v>50</v>
       </c>
       <c r="AS11" s="28" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="AT11" s="28" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="AU11" s="28" t="s">
         <v>67</v>
@@ -3489,7 +3474,7 @@
         <v>1</v>
       </c>
       <c r="AX11" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AY11">
         <v>1</v>
@@ -3501,7 +3486,7 @@
         <v>300</v>
       </c>
       <c r="BB11" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="12" spans="1:54">
@@ -3515,14 +3500,14 @@
         <v>70</v>
       </c>
       <c r="D12" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E12" s="2">
         <v>19447</v>
       </c>
       <c r="F12" s="18">
         <f t="shared" ca="1" si="0"/>
-        <v>72.922222222222217</v>
+        <v>72.924999999999997</v>
       </c>
       <c r="G12" s="5">
         <v>19.13</v>
@@ -3618,13 +3603,13 @@
         <v>1</v>
       </c>
       <c r="AM12" s="3" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="AN12" s="6" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="AO12" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="AP12">
         <v>0</v>
@@ -3662,17 +3647,17 @@
         <v>44251</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="D13" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E13" s="2">
         <v>22058</v>
       </c>
       <c r="F13" s="18">
         <f t="shared" ca="1" si="0"/>
-        <v>65.775000000000006</v>
+        <v>65.777777777777771</v>
       </c>
       <c r="G13" s="5">
         <v>21.48</v>
@@ -3699,7 +3684,7 @@
         <v>0</v>
       </c>
       <c r="P13" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="Q13" s="3">
         <v>1</v>
@@ -3768,13 +3753,13 @@
         <v>0</v>
       </c>
       <c r="AM13" s="3" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="AN13" s="6" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="AO13" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="AP13">
         <v>0</v>
@@ -3786,7 +3771,7 @@
         <v>54</v>
       </c>
       <c r="AS13" s="30" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AV13">
         <v>0</v>
@@ -3795,7 +3780,7 @@
         <v>1</v>
       </c>
       <c r="AX13" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AY13">
         <v>1</v>
@@ -3818,17 +3803,17 @@
         <v>44321</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="D14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E14" s="2">
         <v>24201</v>
       </c>
       <c r="F14" s="18">
         <f t="shared" ca="1" si="0"/>
-        <v>59.908333333333331</v>
+        <v>59.911111111111111</v>
       </c>
       <c r="G14" s="5">
         <v>23.63</v>
@@ -3837,7 +3822,7 @@
         <v>45</v>
       </c>
       <c r="I14" s="23" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="J14">
         <v>0</v>
@@ -3900,22 +3885,22 @@
         <v>1</v>
       </c>
       <c r="AE14" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AF14" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AG14" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AH14" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AI14" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AJ14" s="25" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AK14" s="3">
         <v>2</v>
@@ -3924,13 +3909,13 @@
         <v>0</v>
       </c>
       <c r="AM14" s="26" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AN14" s="6" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AO14" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AP14">
         <v>0</v>
@@ -3948,7 +3933,7 @@
         <v>1</v>
       </c>
       <c r="AX14" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="AY14">
         <v>0</v>
@@ -3971,17 +3956,17 @@
         <v>44335</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="D15" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E15" s="2">
         <v>30784</v>
       </c>
       <c r="F15" s="18">
         <f t="shared" ca="1" si="0"/>
-        <v>41.886111111111113</v>
+        <v>41.888888888888886</v>
       </c>
       <c r="G15" s="5">
         <v>23.65</v>
@@ -4068,7 +4053,7 @@
         <v>0</v>
       </c>
       <c r="AJ15" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="AK15" s="3">
         <v>2</v>
@@ -4077,13 +4062,13 @@
         <v>1</v>
       </c>
       <c r="AM15" s="26" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="AN15" s="6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="AO15" s="6" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="AP15">
         <v>0</v>
@@ -4095,10 +4080,10 @@
         <v>50</v>
       </c>
       <c r="AS15" s="28" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="AT15" s="28" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AV15">
         <v>0</v>
@@ -4107,7 +4092,7 @@
         <v>1</v>
       </c>
       <c r="AX15" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="AY15">
         <v>1</v>
@@ -4130,17 +4115,17 @@
         <v>22</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="D16" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E16" s="2">
         <v>24041</v>
       </c>
       <c r="F16" s="18">
         <f t="shared" ca="1" si="0"/>
-        <v>60.347222222222221</v>
+        <v>60.35</v>
       </c>
       <c r="G16" s="5">
         <v>21.3</v>
@@ -4167,7 +4152,7 @@
         <v>1</v>
       </c>
       <c r="P16" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="Q16" s="3">
         <v>1</v>
@@ -4233,10 +4218,10 @@
         <v>1</v>
       </c>
       <c r="AM16" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="AN16" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="AP16">
         <v>0</v>
@@ -4248,10 +4233,10 @@
         <v>50</v>
       </c>
       <c r="AS16" s="28" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="AT16" s="28" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AV16">
         <v>0</v>
@@ -4260,7 +4245,7 @@
         <v>1</v>
       </c>
       <c r="AX16" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="AY16">
         <v>0</v>
@@ -4283,17 +4268,17 @@
         <v>44512</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="D17" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E17" s="2">
         <v>27390</v>
       </c>
       <c r="F17" s="18">
         <f t="shared" ca="1" si="0"/>
-        <v>51.177777777777777</v>
+        <v>51.180555555555557</v>
       </c>
       <c r="G17" s="5">
         <v>21.7</v>
@@ -4320,7 +4305,7 @@
         <v>1</v>
       </c>
       <c r="P17" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="Q17" s="3">
         <v>1</v>
@@ -4392,7 +4377,7 @@
         <v>0</v>
       </c>
       <c r="AO17" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="AP17">
         <v>0</v>
@@ -4410,7 +4395,7 @@
         <v>1</v>
       </c>
       <c r="AX17" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AY17">
         <v>1</v>
@@ -4436,14 +4421,14 @@
         <v>70</v>
       </c>
       <c r="D18" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E18" s="2">
         <v>23082</v>
       </c>
       <c r="F18" s="18">
         <f t="shared" ca="1" si="0"/>
-        <v>62.969444444444441</v>
+        <v>62.972222222222221</v>
       </c>
       <c r="G18" s="5">
         <v>25.34</v>
@@ -4461,7 +4446,7 @@
         <v>0</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="N18">
         <v>0</v>
@@ -4470,7 +4455,7 @@
         <v>1</v>
       </c>
       <c r="P18" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="Q18" s="3">
         <v>0</v>
@@ -4539,13 +4524,13 @@
         <v>0</v>
       </c>
       <c r="AM18" s="26" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="AN18" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AO18" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="AP18">
         <v>0</v>
@@ -4577,23 +4562,23 @@
     </row>
     <row r="19" spans="1:54">
       <c r="A19" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="B19" s="2">
         <v>44617</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="D19" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="E19" s="2">
         <v>23630</v>
       </c>
       <c r="F19" s="18">
         <f t="shared" ca="1" si="0"/>
-        <v>61.475000000000001</v>
+        <v>61.477777777777774</v>
       </c>
       <c r="G19" s="5">
         <v>24.41</v>
@@ -4680,7 +4665,7 @@
         <v>0</v>
       </c>
       <c r="AJ19" s="3" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="AK19" s="3">
         <v>2</v>
@@ -4689,13 +4674,13 @@
         <v>2</v>
       </c>
       <c r="AM19" s="26" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="AN19" s="6" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="AO19" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="AP19">
         <v>0</v>
@@ -4716,7 +4701,7 @@
         <v>1</v>
       </c>
       <c r="AX19" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="AY19">
         <v>1</v>
@@ -4742,14 +4727,14 @@
         <v>61</v>
       </c>
       <c r="D20" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="E20" s="2">
         <v>21495</v>
       </c>
       <c r="F20" s="18">
         <f t="shared" ca="1" si="0"/>
-        <v>67.319444444444443</v>
+        <v>67.322222222222223</v>
       </c>
       <c r="G20" s="5">
         <v>32.81</v>
@@ -4833,25 +4818,25 @@
         <v>1</v>
       </c>
       <c r="AI20" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="AJ20" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="AK20" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL20" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM20" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN20" s="7" t="s">
+        <v>252</v>
+      </c>
+      <c r="AO20" t="s">
         <v>111</v>
-      </c>
-      <c r="AJ20" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="AK20" s="3">
-        <v>0</v>
-      </c>
-      <c r="AL20" s="3">
-        <v>0</v>
-      </c>
-      <c r="AM20" s="3">
-        <v>0</v>
-      </c>
-      <c r="AN20" s="7" t="s">
-        <v>257</v>
-      </c>
-      <c r="AO20" t="s">
-        <v>112</v>
       </c>
       <c r="AP20">
         <v>0</v>
@@ -4863,10 +4848,10 @@
         <v>50</v>
       </c>
       <c r="AS20" s="28" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="AV20" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="AW20" s="28">
         <v>0</v>
@@ -4992,7 +4977,7 @@
         <v>18</v>
       </c>
       <c r="D1" s="22" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="E1" s="9" t="s">
         <v>20</v>
@@ -5028,7 +5013,7 @@
         <v>78</v>
       </c>
       <c r="P1" s="24" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="Q1" s="22" t="s">
         <v>6</v>
@@ -5046,7 +5031,7 @@
         <v>3</v>
       </c>
       <c r="V1" s="22" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="W1" s="22" t="s">
         <v>41</v>
@@ -5058,19 +5043,19 @@
         <v>42</v>
       </c>
       <c r="Z1" s="22" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="AA1" s="22" t="s">
         <v>24</v>
       </c>
       <c r="AB1" s="22" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="AC1" s="22" t="s">
         <v>43</v>
       </c>
       <c r="AD1" s="22" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="AE1" s="22" t="s">
         <v>11</v>
@@ -5079,7 +5064,7 @@
         <v>60</v>
       </c>
       <c r="AG1" s="22" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="AH1" s="22" t="s">
         <v>28</v>
@@ -5175,7 +5160,7 @@
       </c>
       <c r="G2" s="5">
         <f ca="1">YEARFRAC(F2,TODAY())</f>
-        <v>57.866666666666667</v>
+        <v>57.869444444444447</v>
       </c>
       <c r="H2" s="5">
         <v>25.01</v>
@@ -5343,7 +5328,7 @@
       </c>
       <c r="G3" s="5">
         <f t="shared" ref="G3:G30" ca="1" si="0">YEARFRAC(F3,TODAY())</f>
-        <v>77.352777777777774</v>
+        <v>77.355555555555554</v>
       </c>
       <c r="H3" s="5">
         <v>26.44</v>
@@ -5511,7 +5496,7 @@
       </c>
       <c r="G4" s="5">
         <f t="shared" ca="1" si="0"/>
-        <v>41.213888888888889</v>
+        <v>41.216666666666669</v>
       </c>
       <c r="H4" s="5">
         <v>21.68</v>
@@ -5607,7 +5592,7 @@
         <v>0</v>
       </c>
       <c r="AN4" s="26" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AO4" s="7" t="s">
         <v>68</v>
@@ -5666,7 +5651,7 @@
         <v>44244</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>73</v>
@@ -5676,7 +5661,7 @@
       </c>
       <c r="G5" s="5">
         <f t="shared" ca="1" si="0"/>
-        <v>54.591666666666669</v>
+        <v>54.594444444444441</v>
       </c>
       <c r="H5" s="5">
         <v>18.21</v>
@@ -5772,7 +5757,7 @@
         <v>0</v>
       </c>
       <c r="AN5" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="AO5" s="6" t="s">
         <v>72</v>
@@ -5796,7 +5781,7 @@
         <v>75</v>
       </c>
       <c r="AV5" s="35" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="AW5">
         <v>1</v>
@@ -5837,7 +5822,7 @@
         <v>44026</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>81</v>
@@ -5847,7 +5832,7 @@
       </c>
       <c r="G6" s="5">
         <f t="shared" ca="1" si="0"/>
-        <v>46.06111111111111</v>
+        <v>46.06388888888889</v>
       </c>
       <c r="H6" s="5">
         <v>25.55</v>
@@ -5943,7 +5928,7 @@
         <v>1</v>
       </c>
       <c r="AN6" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AO6" t="s">
         <v>80</v>
@@ -5999,14 +5984,14 @@
         <v>70</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F7" s="2">
         <v>28651</v>
       </c>
       <c r="G7" s="5">
         <f t="shared" ca="1" si="0"/>
-        <v>47.725000000000001</v>
+        <v>47.727777777777774</v>
       </c>
       <c r="H7" s="5">
         <v>24.34</v>
@@ -6015,7 +6000,7 @@
         <v>45</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="K7">
         <v>0</v>
@@ -6093,7 +6078,7 @@
         <v>0</v>
       </c>
       <c r="AK7" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AL7" s="3">
         <v>2</v>
@@ -6105,10 +6090,10 @@
         <v>0</v>
       </c>
       <c r="AO7" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AP7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AQ7">
         <v>0</v>
@@ -6126,7 +6111,7 @@
         <v>1</v>
       </c>
       <c r="AY7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AZ7">
         <v>1</v>
@@ -6140,8 +6125,8 @@
       <c r="BC7" s="35">
         <v>400</v>
       </c>
-      <c r="BD7" s="35" t="s">
-        <v>84</v>
+      <c r="BD7" s="35">
+        <v>350</v>
       </c>
       <c r="BE7" t="s">
         <v>83</v>
@@ -6161,14 +6146,14 @@
         <v>70</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F8" s="2">
         <v>24762</v>
       </c>
       <c r="G8" s="5">
         <f t="shared" ca="1" si="0"/>
-        <v>58.37222222222222</v>
+        <v>58.375</v>
       </c>
       <c r="H8" s="5">
         <v>22.1</v>
@@ -6255,7 +6240,7 @@
         <v>0</v>
       </c>
       <c r="AK8" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AL8" s="3">
         <v>2</v>
@@ -6264,13 +6249,13 @@
         <v>1</v>
       </c>
       <c r="AN8" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AO8" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="AP8" t="s">
         <v>90</v>
-      </c>
-      <c r="AP8" t="s">
-        <v>91</v>
       </c>
       <c r="AQ8">
         <v>0</v>
@@ -6323,14 +6308,14 @@
         <v>70</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F9" s="2">
         <v>24595</v>
       </c>
       <c r="G9" s="5">
         <f t="shared" ca="1" si="0"/>
-        <v>58.827777777777776</v>
+        <v>58.830555555555556</v>
       </c>
       <c r="H9" s="5">
         <v>23.49</v>
@@ -6426,13 +6411,13 @@
         <v>0</v>
       </c>
       <c r="AN9" s="26" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="AO9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="AP9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="AQ9">
         <v>0</v>
@@ -6444,13 +6429,13 @@
         <v>50</v>
       </c>
       <c r="AT9" s="35" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="AU9" s="35" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="AV9" s="35" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="AW9">
         <v>0</v>
@@ -6491,14 +6476,14 @@
         <v>70</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F10" s="2">
         <v>24240</v>
       </c>
       <c r="G10" s="5">
         <f t="shared" ca="1" si="0"/>
-        <v>59.8</v>
+        <v>59.802777777777777</v>
       </c>
       <c r="H10" s="5">
         <v>30.61</v>
@@ -6594,13 +6579,13 @@
         <v>0</v>
       </c>
       <c r="AN10" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="AO10" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="AP10" s="8" t="s">
         <v>103</v>
-      </c>
-      <c r="AP10" s="8" t="s">
-        <v>104</v>
       </c>
       <c r="AQ10">
         <v>0</v>
@@ -6650,14 +6635,14 @@
         <v>61</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F11" s="2">
         <v>26926</v>
       </c>
       <c r="G11" s="5">
         <f t="shared" ca="1" si="0"/>
-        <v>52.45</v>
+        <v>52.452777777777776</v>
       </c>
       <c r="H11" s="5">
         <v>30.72</v>
@@ -6684,7 +6669,7 @@
         <v>0</v>
       </c>
       <c r="Q11" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="R11" s="3">
         <v>1</v>
@@ -6744,7 +6729,7 @@
         <v>1</v>
       </c>
       <c r="AK11" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AL11" s="3">
         <v>0</v>
@@ -6753,13 +6738,13 @@
         <v>0</v>
       </c>
       <c r="AN11" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AO11" s="6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="AP11" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="AQ11">
         <v>0</v>
@@ -6771,10 +6756,10 @@
         <v>50</v>
       </c>
       <c r="AT11" s="35" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="AU11" s="35" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="AW11">
         <v>0</v>
@@ -6783,7 +6768,7 @@
         <v>1</v>
       </c>
       <c r="AY11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="AZ11">
         <v>0</v>
@@ -6818,14 +6803,14 @@
         <v>70</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F12" s="2">
         <v>34325</v>
       </c>
       <c r="G12" s="5">
         <f t="shared" ca="1" si="0"/>
-        <v>32.19166666666667</v>
+        <v>32.194444444444443</v>
       </c>
       <c r="H12" s="5">
         <v>20.9</v>
@@ -6834,7 +6819,7 @@
         <v>45</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="K12">
         <v>0</v>
@@ -6855,7 +6840,7 @@
         <v>0</v>
       </c>
       <c r="R12" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S12" s="3">
         <v>1</v>
@@ -6912,7 +6897,7 @@
         <v>1</v>
       </c>
       <c r="AK12" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AL12" s="3">
         <v>2</v>
@@ -6921,13 +6906,13 @@
         <v>1</v>
       </c>
       <c r="AN12" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="AO12" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="AP12" t="s">
         <v>172</v>
-      </c>
-      <c r="AO12" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="AP12" t="s">
-        <v>173</v>
       </c>
       <c r="AQ12">
         <v>0</v>
@@ -6939,13 +6924,13 @@
         <v>50</v>
       </c>
       <c r="AT12" s="35" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="AU12" s="35" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="AV12" s="35" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="AW12">
         <v>0</v>
@@ -6954,7 +6939,7 @@
         <v>1</v>
       </c>
       <c r="AY12" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AZ12">
         <v>1</v>
@@ -6968,8 +6953,8 @@
       <c r="BC12" s="35">
         <v>50</v>
       </c>
-      <c r="BD12" s="35" t="s">
-        <v>175</v>
+      <c r="BD12" s="35">
+        <v>282</v>
       </c>
       <c r="BE12" t="s">
         <v>77</v>
@@ -6989,14 +6974,14 @@
         <v>70</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F13" s="2">
         <v>29223</v>
       </c>
       <c r="G13" s="5">
         <f t="shared" ca="1" si="0"/>
-        <v>46.161111111111111</v>
+        <v>46.163888888888891</v>
       </c>
       <c r="H13" s="5">
         <v>23.96</v>
@@ -7005,7 +6990,7 @@
         <v>45</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="K13">
         <v>0</v>
@@ -7023,7 +7008,7 @@
         <v>0</v>
       </c>
       <c r="Q13" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="R13" s="3">
         <v>0</v>
@@ -7092,13 +7077,13 @@
         <v>0</v>
       </c>
       <c r="AN13" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="AO13" s="6" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="AP13" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="AQ13">
         <v>0</v>
@@ -7127,8 +7112,8 @@
       <c r="BC13" s="35">
         <v>60</v>
       </c>
-      <c r="BD13" s="35" t="s">
-        <v>178</v>
+      <c r="BD13" s="35">
+        <v>350</v>
       </c>
       <c r="BE13" t="s">
         <v>77</v>
@@ -7148,14 +7133,14 @@
         <v>70</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F14" s="2">
         <v>31562</v>
       </c>
       <c r="G14" s="5">
         <f t="shared" ca="1" si="0"/>
-        <v>39.75277777777778</v>
+        <v>39.755555555555553</v>
       </c>
       <c r="H14" s="5">
         <v>19.309999999999999</v>
@@ -7164,7 +7149,7 @@
         <v>45</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="K14">
         <v>0</v>
@@ -7239,7 +7224,7 @@
         <v>0</v>
       </c>
       <c r="AK14" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AL14" s="3">
         <v>2</v>
@@ -7248,13 +7233,13 @@
         <v>0</v>
       </c>
       <c r="AN14" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="AO14" s="6" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="AP14" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="AQ14">
         <v>0</v>
@@ -7266,7 +7251,7 @@
         <v>50</v>
       </c>
       <c r="AT14" s="35" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="AW14">
         <v>1</v>
@@ -7275,7 +7260,7 @@
         <v>1</v>
       </c>
       <c r="AY14" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="AZ14">
         <v>1</v>
@@ -7310,14 +7295,14 @@
         <v>70</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F15" s="2">
         <v>27291</v>
       </c>
       <c r="G15" s="5">
         <f t="shared" ca="1" si="0"/>
-        <v>51.45</v>
+        <v>51.452777777777776</v>
       </c>
       <c r="H15" s="5">
         <v>18.54</v>
@@ -7404,7 +7389,7 @@
         <v>0</v>
       </c>
       <c r="AK15" s="3" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="AL15" s="3">
         <v>2</v>
@@ -7413,13 +7398,13 @@
         <v>1</v>
       </c>
       <c r="AN15" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AO15" s="6" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="AP15" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="AQ15">
         <v>0</v>
@@ -7431,7 +7416,7 @@
         <v>54</v>
       </c>
       <c r="AT15" s="35" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="AW15">
         <v>0</v>
@@ -7472,14 +7457,14 @@
         <v>70</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F16" s="2">
         <v>28651</v>
       </c>
       <c r="G16" s="5">
         <f t="shared" ca="1" si="0"/>
-        <v>47.725000000000001</v>
+        <v>47.727777777777774</v>
       </c>
       <c r="H16" s="5">
         <v>24.34</v>
@@ -7488,7 +7473,7 @@
         <v>45</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="K16">
         <v>0</v>
@@ -7566,7 +7551,7 @@
         <v>0</v>
       </c>
       <c r="AK16" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AL16" s="3">
         <v>2</v>
@@ -7578,10 +7563,10 @@
         <v>0</v>
       </c>
       <c r="AO16" s="6" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="AP16" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="AQ16">
         <v>0</v>
@@ -7593,7 +7578,7 @@
         <v>50</v>
       </c>
       <c r="AT16" s="35" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="AW16">
         <v>0</v>
@@ -7602,7 +7587,7 @@
         <v>1</v>
       </c>
       <c r="AY16" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="AZ16">
         <v>1</v>
@@ -7616,14 +7601,14 @@
       <c r="BC16" s="35">
         <v>400</v>
       </c>
-      <c r="BD16" s="35" t="s">
-        <v>189</v>
+      <c r="BD16" s="35">
+        <v>350</v>
       </c>
       <c r="BE16" t="s">
         <v>77</v>
       </c>
       <c r="BF16" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
     <row r="17" spans="1:57">
@@ -7640,14 +7625,14 @@
         <v>61</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="F17" s="2">
         <v>19534</v>
       </c>
       <c r="G17" s="5">
         <f t="shared" ca="1" si="0"/>
-        <v>72.686111111111117</v>
+        <v>72.688888888888883</v>
       </c>
       <c r="H17" s="5">
         <v>30.86</v>
@@ -7674,7 +7659,7 @@
         <v>0</v>
       </c>
       <c r="Q17" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="R17" s="3">
         <v>1</v>
@@ -7734,7 +7719,7 @@
         <v>0</v>
       </c>
       <c r="AK17" s="3" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="AL17" s="3">
         <v>1</v>
@@ -7749,7 +7734,7 @@
         <v>62</v>
       </c>
       <c r="AP17" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="AQ17">
         <v>0</v>
@@ -7799,14 +7784,14 @@
         <v>61</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="F18" s="2">
         <v>17617</v>
       </c>
       <c r="G18" s="5">
         <f t="shared" ca="1" si="0"/>
-        <v>77.933333333333337</v>
+        <v>77.936111111111117</v>
       </c>
       <c r="H18" s="5">
         <v>26.85</v>
@@ -7836,7 +7821,7 @@
         <v>0</v>
       </c>
       <c r="R18" s="3" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="S18" s="3">
         <v>1</v>
@@ -7902,13 +7887,13 @@
         <v>1</v>
       </c>
       <c r="AN18" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AO18" s="6" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="AP18" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="AR18" s="34">
         <v>45071</v>
@@ -7917,13 +7902,13 @@
         <v>50</v>
       </c>
       <c r="AT18" s="35" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="AU18" s="35" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="AV18" s="35" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AW18">
         <v>1</v>
@@ -7961,17 +7946,17 @@
         <v>44292</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="E19" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="F19" s="2">
         <v>28642</v>
       </c>
       <c r="G19" s="5">
         <f t="shared" ca="1" si="0"/>
-        <v>47.75</v>
+        <v>47.75277777777778</v>
       </c>
       <c r="H19" s="5">
         <v>22.43</v>
@@ -8067,13 +8052,13 @@
         <v>1</v>
       </c>
       <c r="AN19" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="AO19" s="6" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="AP19" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="AQ19">
         <v>0</v>
@@ -8120,17 +8105,17 @@
         <v>44258</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="F20" s="2">
         <v>16837</v>
       </c>
       <c r="G20" s="5">
         <f t="shared" ca="1" si="0"/>
-        <v>80.075000000000003</v>
+        <v>80.077777777777783</v>
       </c>
       <c r="H20" s="5">
         <v>33.020000000000003</v>
@@ -8139,7 +8124,7 @@
         <v>45</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="K20">
         <v>1</v>
@@ -8160,7 +8145,7 @@
         <v>0</v>
       </c>
       <c r="Q20" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="R20" s="3">
         <v>1</v>
@@ -8220,7 +8205,7 @@
         <v>0</v>
       </c>
       <c r="AK20" s="3" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="AL20" s="3">
         <v>1</v>
@@ -8232,10 +8217,10 @@
         <v>0</v>
       </c>
       <c r="AO20" s="7" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="AP20" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="AQ20">
         <v>0</v>
@@ -8247,7 +8232,7 @@
         <v>54</v>
       </c>
       <c r="AT20" s="35" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="AW20">
         <v>0</v>
@@ -8276,7 +8261,7 @@
     </row>
     <row r="21" spans="1:57">
       <c r="A21" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B21" s="2">
         <v>44113</v>
@@ -8285,17 +8270,17 @@
         <v>44167</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="F21" s="2">
         <v>27665</v>
       </c>
       <c r="G21" s="5">
         <f t="shared" ca="1" si="0"/>
-        <v>50.424999999999997</v>
+        <v>50.427777777777777</v>
       </c>
       <c r="H21" s="5">
         <v>18.989999999999998</v>
@@ -8373,31 +8358,31 @@
         <v>0</v>
       </c>
       <c r="AH21" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AI21" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AJ21" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AK21" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AL21" s="3">
         <v>2</v>
       </c>
       <c r="AM21" s="25" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AN21" s="25" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AO21" s="16" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AP21" s="16" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AQ21">
         <v>0</v>
@@ -8412,10 +8397,10 @@
         <v>67</v>
       </c>
       <c r="AU21" s="35" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AV21" s="35" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="AW21">
         <v>0</v>
@@ -8424,7 +8409,7 @@
         <v>1</v>
       </c>
       <c r="AY21" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="AZ21">
         <v>0</v>
@@ -8447,7 +8432,7 @@
     </row>
     <row r="22" spans="1:57">
       <c r="A22" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B22" s="2">
         <v>44148</v>
@@ -8456,17 +8441,17 @@
         <v>44217</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="F22" s="2">
         <v>34886</v>
       </c>
       <c r="G22" s="5">
         <f t="shared" ca="1" si="0"/>
-        <v>30.652777777777779</v>
+        <v>30.655555555555555</v>
       </c>
       <c r="H22" s="5">
         <v>22.5</v>
@@ -8493,7 +8478,7 @@
         <v>0</v>
       </c>
       <c r="Q22" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="R22" s="3">
         <v>1</v>
@@ -8544,31 +8529,31 @@
         <v>0</v>
       </c>
       <c r="AH22" s="25" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AI22" s="25" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AJ22" s="25" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AK22" s="25" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AL22" s="3">
         <v>2</v>
       </c>
       <c r="AM22" s="25" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AN22" s="25" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AO22" s="16" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AP22" s="16" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AQ22">
         <v>0</v>
@@ -8618,14 +8603,14 @@
         <v>70</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F23" s="2">
         <v>28867</v>
       </c>
       <c r="G23" s="5">
         <f t="shared" ca="1" si="0"/>
-        <v>47.136111111111113</v>
+        <v>47.138888888888886</v>
       </c>
       <c r="H23" s="5">
         <v>26</v>
@@ -8652,7 +8637,7 @@
         <v>0</v>
       </c>
       <c r="Q23" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="R23" s="3">
         <v>1</v>
@@ -8712,7 +8697,7 @@
         <v>0</v>
       </c>
       <c r="AK23" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AL23" s="3">
         <v>2</v>
@@ -8721,13 +8706,13 @@
         <v>0</v>
       </c>
       <c r="AN23" s="26" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AO23" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="AP23" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="AQ23">
         <v>0</v>
@@ -8739,7 +8724,7 @@
         <v>54</v>
       </c>
       <c r="AT23" s="35" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="AW23">
         <v>0</v>
@@ -8777,17 +8762,17 @@
         <v>44344</v>
       </c>
       <c r="D24" s="23" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="F24" s="2">
         <v>23180</v>
       </c>
       <c r="G24" s="5">
         <f t="shared" ca="1" si="0"/>
-        <v>62.702777777777776</v>
+        <v>62.705555555555556</v>
       </c>
       <c r="H24" s="5">
         <v>28.15</v>
@@ -8874,7 +8859,7 @@
         <v>0</v>
       </c>
       <c r="AK24" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="AL24" s="3">
         <v>2</v>
@@ -8883,13 +8868,13 @@
         <v>0</v>
       </c>
       <c r="AN24" s="26" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="AO24" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="AP24" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="AQ24">
         <v>0</v>
@@ -8901,7 +8886,7 @@
         <v>50</v>
       </c>
       <c r="AT24" s="35" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="AW24">
         <v>0</v>
@@ -8910,13 +8895,13 @@
         <v>1</v>
       </c>
       <c r="AY24" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="AZ24">
         <v>1</v>
       </c>
       <c r="BA24" s="35" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="BB24" s="35">
         <v>750</v>
@@ -8945,14 +8930,14 @@
         <v>70</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F25" s="2">
         <v>15710</v>
       </c>
       <c r="G25" s="5">
         <f t="shared" ca="1" si="0"/>
-        <v>83.158333333333331</v>
+        <v>83.161111111111111</v>
       </c>
       <c r="H25" s="5">
         <v>22.67</v>
@@ -9039,7 +9024,7 @@
         <v>1</v>
       </c>
       <c r="AK25" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AL25" s="3">
         <v>0</v>
@@ -9048,13 +9033,13 @@
         <v>0</v>
       </c>
       <c r="AN25" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AO25" s="6" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="AP25" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="AR25" s="34">
         <v>45790</v>
@@ -9063,7 +9048,7 @@
         <v>54</v>
       </c>
       <c r="AT25" s="35" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="AW25">
         <v>1</v>
@@ -9104,14 +9089,14 @@
         <v>70</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F26" s="2">
         <v>24240</v>
       </c>
       <c r="G26" s="5">
         <f t="shared" ca="1" si="0"/>
-        <v>59.8</v>
+        <v>59.802777777777777</v>
       </c>
       <c r="H26" s="5">
         <v>30.61</v>
@@ -9210,10 +9195,10 @@
         <v>0</v>
       </c>
       <c r="AO26" s="6" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="AP26" s="6" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="AQ26">
         <v>0</v>
@@ -9242,8 +9227,8 @@
       <c r="BB26" s="35">
         <v>550</v>
       </c>
-      <c r="BC26" s="35" t="s">
-        <v>216</v>
+      <c r="BC26" s="35">
+        <v>250</v>
       </c>
       <c r="BD26" s="35">
         <v>400</v>
@@ -9266,14 +9251,14 @@
         <v>70</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F27" s="2">
         <v>27346</v>
       </c>
       <c r="G27" s="5">
         <f t="shared" ca="1" si="0"/>
-        <v>51.3</v>
+        <v>51.302777777777777</v>
       </c>
       <c r="H27" s="5">
         <v>26.28</v>
@@ -9300,7 +9285,7 @@
         <v>0</v>
       </c>
       <c r="Q27" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="R27" s="3">
         <v>1</v>
@@ -9360,7 +9345,7 @@
         <v>0</v>
       </c>
       <c r="AK27" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AL27" s="3">
         <v>2</v>
@@ -9369,13 +9354,13 @@
         <v>1</v>
       </c>
       <c r="AN27" s="26" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="AO27" s="6" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="AP27" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="AQ27">
         <v>0</v>
@@ -9387,10 +9372,10 @@
         <v>54</v>
       </c>
       <c r="AT27" s="35" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="AU27" s="35" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="AW27">
         <v>1</v>
@@ -9431,14 +9416,14 @@
         <v>70</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="F28" s="2">
         <v>30196</v>
       </c>
       <c r="G28" s="5">
         <f t="shared" ca="1" si="0"/>
-        <v>43.49722222222222</v>
+        <v>43.5</v>
       </c>
       <c r="H28" s="5">
         <v>27.84</v>
@@ -9465,7 +9450,7 @@
         <v>0</v>
       </c>
       <c r="Q28" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="R28" s="3">
         <v>1</v>
@@ -9477,7 +9462,7 @@
         <v>0</v>
       </c>
       <c r="U28" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="V28" s="3">
         <v>0</v>
@@ -9534,13 +9519,13 @@
         <v>0</v>
       </c>
       <c r="AN28" s="26" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="AO28" s="6" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="AP28" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="AQ28">
         <v>0</v>
@@ -9552,7 +9537,7 @@
         <v>50</v>
       </c>
       <c r="AT28" s="35" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="AW28">
         <v>0</v>
@@ -9561,7 +9546,7 @@
         <v>1</v>
       </c>
       <c r="AY28" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="AZ28">
         <v>0</v>
@@ -9596,14 +9581,14 @@
         <v>70</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F29" s="2">
         <v>30387</v>
       </c>
       <c r="G29" s="5">
         <f t="shared" ca="1" si="0"/>
-        <v>42.969444444444441</v>
+        <v>42.972222222222221</v>
       </c>
       <c r="H29" s="5">
         <v>27.25</v>
@@ -9630,7 +9615,7 @@
         <v>0</v>
       </c>
       <c r="Q29" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="R29" s="3">
         <v>1</v>
@@ -9690,7 +9675,7 @@
         <v>0</v>
       </c>
       <c r="AK29" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AL29" s="3">
         <v>2</v>
@@ -9699,13 +9684,13 @@
         <v>0</v>
       </c>
       <c r="AN29" s="26" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AO29" s="6" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="AP29" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="AQ29">
         <v>0</v>
@@ -9752,17 +9737,17 @@
         <v>44123</v>
       </c>
       <c r="D30" s="23" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="F30" s="2">
         <v>24627</v>
       </c>
       <c r="G30" s="5">
         <f t="shared" ca="1" si="0"/>
-        <v>58.741666666666667</v>
+        <v>58.744444444444447</v>
       </c>
       <c r="H30" s="5">
         <v>19.13</v>
@@ -9789,7 +9774,7 @@
         <v>0</v>
       </c>
       <c r="Q30" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="R30" s="3">
         <v>0</v>
@@ -9858,13 +9843,13 @@
         <v>0</v>
       </c>
       <c r="AN30" s="26" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AO30" s="6" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="AP30" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="AQ30">
         <v>0</v>
@@ -9876,10 +9861,10 @@
         <v>50</v>
       </c>
       <c r="AT30" s="35" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="AU30" s="35" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="AV30" s="35" t="s">
         <v>63</v>
@@ -9891,7 +9876,7 @@
         <v>1</v>
       </c>
       <c r="AY30" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="AZ30">
         <v>1</v>

</xml_diff>